<commit_message>
Added more tools and updated excel
</commit_message>
<xml_diff>
--- a/fault_codes.xlsx
+++ b/fault_codes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyank_SH\OneDrive\Desktop\RVU\Hackathons\sentinal_hack_ksit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\Hackathons\Sentinel_Hack\Team_MLFSS-SentinelHack\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D63C31-E429-407D-BF21-CD6C80CFC2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7043DB6E-7AEA-4E16-B004-8218288D1E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{928AC3C0-4CDD-4784-92DB-26296861BEEF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{928AC3C0-4CDD-4784-92DB-26296861BEEF}"/>
   </bookViews>
   <sheets>
     <sheet name="fault_codes" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="194">
   <si>
     <t>Code</t>
   </si>
@@ -446,6 +446,177 @@
   </si>
   <si>
     <t>Independent line pressure check</t>
+  </si>
+  <si>
+    <t>Digital Manometer</t>
+  </si>
+  <si>
+    <t>Filter Housing Wrench Set</t>
+  </si>
+  <si>
+    <t>Compressed Air Gun</t>
+  </si>
+  <si>
+    <t>Torque Wrench (50-150 Nm)</t>
+  </si>
+  <si>
+    <t>Spark Plug Socket Set</t>
+  </si>
+  <si>
+    <t>Torque Wrench (25-35 Nm)</t>
+  </si>
+  <si>
+    <t>Feeler Gauge Set</t>
+  </si>
+  <si>
+    <t>Anti-Seize Compound</t>
+  </si>
+  <si>
+    <t>Fuel System Pressure Tester</t>
+  </si>
+  <si>
+    <t>Electronic Timing Light</t>
+  </si>
+  <si>
+    <t>Fuel Line Disconnect Tools</t>
+  </si>
+  <si>
+    <t>Bearing Puller Set</t>
+  </si>
+  <si>
+    <t>Hydraulic Press</t>
+  </si>
+  <si>
+    <t>Dial Indicator</t>
+  </si>
+  <si>
+    <t>Coolant System Flush Kit</t>
+  </si>
+  <si>
+    <t>Torque Wrench (120-180 Nm)</t>
+  </si>
+  <si>
+    <t>Engine Hoist (5-ton capacity)</t>
+  </si>
+  <si>
+    <t>Cylinder Bore Gauge</t>
+  </si>
+  <si>
+    <t>Plastigage Kit</t>
+  </si>
+  <si>
+    <t>Ring Compressor Tool</t>
+  </si>
+  <si>
+    <t>Precision Torque Wrench (200-400 Nm)</t>
+  </si>
+  <si>
+    <t>Flange Spreader Tool</t>
+  </si>
+  <si>
+    <t>Thread Compound Applicator</t>
+  </si>
+  <si>
+    <t>Ultrasonic Thickness Gauge</t>
+  </si>
+  <si>
+    <t>Wire Brush Set</t>
+  </si>
+  <si>
+    <t>Sandblasting Equipment</t>
+  </si>
+  <si>
+    <t>Surface Profile Gauge</t>
+  </si>
+  <si>
+    <t>Spray Application Gun</t>
+  </si>
+  <si>
+    <t>Hydraulic Test Pump</t>
+  </si>
+  <si>
+    <t>Valve Spring Compressor</t>
+  </si>
+  <si>
+    <t>Precision Pressure Gauge</t>
+  </si>
+  <si>
+    <t>Torque Multiplier</t>
+  </si>
+  <si>
+    <t>Magnetic Particle Inspection Kit</t>
+  </si>
+  <si>
+    <t>Pipe Alignment Clamps</t>
+  </si>
+  <si>
+    <t>Hydraulic Pipe Cutter</t>
+  </si>
+  <si>
+    <t>Welding Equipment</t>
+  </si>
+  <si>
+    <t>Expansion Joint Installation Tool</t>
+  </si>
+  <si>
+    <t>Emergency Isolation Tools</t>
+  </si>
+  <si>
+    <t>Heavy-Duty Pipe Cutter</t>
+  </si>
+  <si>
+    <t>Hydraulic Lifting Equipment</t>
+  </si>
+  <si>
+    <t>Welding Habitat Enclosure</t>
+  </si>
+  <si>
+    <t>Radiographic Testing Equipment</t>
+  </si>
+  <si>
+    <t>Seal Face Inspection Mirror</t>
+  </si>
+  <si>
+    <t>Precision Feeler Gauges</t>
+  </si>
+  <si>
+    <t>Pump Casing Lifting Sling</t>
+  </si>
+  <si>
+    <t>High-Pressure Water Hose</t>
+  </si>
+  <si>
+    <t>LED Inspection Light</t>
+  </si>
+  <si>
+    <t>Non-Sparking Bronze Scraper</t>
+  </si>
+  <si>
+    <t>Precision Dial Indicators</t>
+  </si>
+  <si>
+    <t>Hydraulic Jack System</t>
+  </si>
+  <si>
+    <t>Impeller Puller Set</t>
+  </si>
+  <si>
+    <t>Thread Locking Compound</t>
+  </si>
+  <si>
+    <t>Surface Roughness Gauge</t>
+  </si>
+  <si>
+    <t>Overhead Crane with 5-Ton Capacity</t>
+  </si>
+  <si>
+    <t>Hydraulic Press Assembly</t>
+  </si>
+  <si>
+    <t>Shaft Alignment Mandrel</t>
+  </si>
+  <si>
+    <t>Precision Measuring Instruments</t>
   </si>
 </sst>
 </file>
@@ -453,9 +624,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,6 +652,26 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -539,20 +730,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -569,12 +748,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -897,370 +1089,370 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A2" s="12">
+      <c r="A2" s="7">
         <v>39083</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A3" s="12">
+      <c r="A3" s="7">
         <v>39114</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A4" s="12">
+      <c r="A4" s="7">
         <v>38412</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="12">
+      <c r="A5" s="7">
         <v>38353</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A6" s="12">
+      <c r="A6" s="7">
         <v>36192</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="5" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A7" s="12">
+      <c r="A7" s="7">
         <v>39084</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A8" s="12">
+      <c r="A8" s="7">
         <v>39115</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A9" s="12">
+      <c r="A9" s="7">
         <v>38413</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A10" s="12">
+      <c r="A10" s="7">
         <v>38354</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="12">
+      <c r="A11" s="7">
         <v>36193</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="12">
+      <c r="A12" s="7">
         <v>39085</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="12">
+      <c r="A13" s="7">
         <v>39116</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="69" x14ac:dyDescent="0.3">
-      <c r="A14" s="12">
+      <c r="A14" s="7">
         <v>38414</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="12">
+      <c r="A15" s="7">
         <v>38355</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="12">
+      <c r="A16" s="7">
         <v>36194</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="5" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1271,307 +1463,882 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0CDD125-B3AF-4A3F-9F17-8AF6172F4405}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.109375" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="24.109375" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="12" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="12" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="69" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="12" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="69" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="12" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:4" ht="75" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:4" ht="75" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="12" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:4" ht="45" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="12" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="69" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="12" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="12" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="12" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:4" ht="90" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="12" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="12" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="69" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:4" ht="75" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="12" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:4" ht="75" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="12" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:4" ht="60" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="12" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:4" ht="90" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="12" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="69" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:4" ht="75" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="12" t="s">
         <v>136</v>
       </c>
+    </row>
+    <row r="22" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+    </row>
+    <row r="23" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+    </row>
+    <row r="25" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+    </row>
+    <row r="26" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+    </row>
+    <row r="27" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+    </row>
+    <row r="28" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+    </row>
+    <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+    </row>
+    <row r="30" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+    </row>
+    <row r="31" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+    </row>
+    <row r="32" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+    </row>
+    <row r="38" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+    </row>
+    <row r="39" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+    </row>
+    <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+    </row>
+    <row r="41" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+    </row>
+    <row r="42" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+    </row>
+    <row r="43" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+    </row>
+    <row r="44" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A44" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+    </row>
+    <row r="45" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+    </row>
+    <row r="46" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+    </row>
+    <row r="47" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A47" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+    </row>
+    <row r="48" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+    </row>
+    <row r="49" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+    </row>
+    <row r="50" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+    </row>
+    <row r="51" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A51" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+    </row>
+    <row r="52" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A52" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" s="13"/>
+      <c r="D52" s="13"/>
+    </row>
+    <row r="53" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+    </row>
+    <row r="54" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A54" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+    </row>
+    <row r="55" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+    </row>
+    <row r="56" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C56" s="13"/>
+      <c r="D56" s="13"/>
+    </row>
+    <row r="57" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C57" s="13"/>
+      <c r="D57" s="13"/>
+    </row>
+    <row r="58" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A58" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+    </row>
+    <row r="59" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A59" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C59" s="13"/>
+      <c r="D59" s="13"/>
+    </row>
+    <row r="60" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C60" s="13"/>
+      <c r="D60" s="13"/>
+    </row>
+    <row r="61" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A61" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B61" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C61" s="13"/>
+      <c r="D61" s="13"/>
+    </row>
+    <row r="62" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A62" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C62" s="13"/>
+      <c r="D62" s="13"/>
+    </row>
+    <row r="63" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A63" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C63" s="13"/>
+      <c r="D63" s="13"/>
+    </row>
+    <row r="64" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A64" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C64" s="13"/>
+      <c r="D64" s="13"/>
+    </row>
+    <row r="65" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A65" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B65" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
+    </row>
+    <row r="66" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A66" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+    </row>
+    <row r="67" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A67" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C67" s="13"/>
+      <c r="D67" s="13"/>
+    </row>
+    <row r="68" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A68" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="B68" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C68" s="13"/>
+      <c r="D68" s="13"/>
+    </row>
+    <row r="69" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A69" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B69" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C69" s="13"/>
+      <c r="D69" s="13"/>
+    </row>
+    <row r="70" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A70" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B70" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C70" s="13"/>
+      <c r="D70" s="13"/>
+    </row>
+    <row r="71" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A71" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B71" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C71" s="13"/>
+      <c r="D71" s="13"/>
+    </row>
+    <row r="72" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B72" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C72" s="13"/>
+      <c r="D72" s="13"/>
+    </row>
+    <row r="73" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A73" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B73" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C73" s="13"/>
+      <c r="D73" s="13"/>
+    </row>
+    <row r="74" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A74" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B74" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C74" s="13"/>
+      <c r="D74" s="13"/>
+    </row>
+    <row r="75" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A75" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="B75" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C75" s="13"/>
+      <c r="D75" s="13"/>
+    </row>
+    <row r="76" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A76" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="B76" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C76" s="13"/>
+      <c r="D76" s="13"/>
+    </row>
+    <row r="77" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A77" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B77" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C77" s="13"/>
+      <c r="D77" s="13"/>
+    </row>
+    <row r="78" spans="1:4" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A78" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B78" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C78" s="13"/>
+      <c r="D78" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>